<commit_message>
add fuses to Dimmer VIN
</commit_message>
<xml_diff>
--- a/IO_Overview.xlsx
+++ b/IO_Overview.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\baischerl\Documents\localProject\cad\RS485-IO-Extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B72E963-36CD-4C13-9C02-B5CDC0F2AC6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{233F62ED-2EB9-40CA-A05A-C290C00C4621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{22052B5C-B221-40B8-A976-D46AAAD19BD0}"/>
+    <workbookView xWindow="29190" yWindow="-7275" windowWidth="28800" windowHeight="15345" xr2:uid="{22052B5C-B221-40B8-A976-D46AAAD19BD0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1753,7 +1753,7 @@
         <v>32</v>
       </c>
       <c r="X65" t="s">
-        <v>104</v>
+        <v>81</v>
       </c>
     </row>
     <row r="66" spans="22:24" x14ac:dyDescent="0.25">
@@ -1762,7 +1762,7 @@
         <v>34</v>
       </c>
       <c r="X66" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="67" spans="22:24" x14ac:dyDescent="0.25">
@@ -1771,7 +1771,7 @@
         <v>37</v>
       </c>
       <c r="X67" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="68" spans="22:24" x14ac:dyDescent="0.25">
@@ -1780,7 +1780,7 @@
         <v>38</v>
       </c>
       <c r="X68" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="69" spans="22:24" x14ac:dyDescent="0.25">
@@ -1789,7 +1789,7 @@
         <v>39</v>
       </c>
       <c r="X69" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
     </row>
     <row r="70" spans="22:24" x14ac:dyDescent="0.25">
@@ -1882,11 +1882,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="V64:V80"/>
-    <mergeCell ref="X72:X73"/>
-    <mergeCell ref="X74:X75"/>
-    <mergeCell ref="X76:X77"/>
-    <mergeCell ref="X78:X79"/>
     <mergeCell ref="V1:V8"/>
     <mergeCell ref="V46:V62"/>
     <mergeCell ref="X54:X55"/>
@@ -1903,6 +1898,11 @@
     <mergeCell ref="X38:X39"/>
     <mergeCell ref="X40:X41"/>
     <mergeCell ref="X42:X43"/>
+    <mergeCell ref="V64:V80"/>
+    <mergeCell ref="X72:X73"/>
+    <mergeCell ref="X74:X75"/>
+    <mergeCell ref="X76:X77"/>
+    <mergeCell ref="X78:X79"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>